<commit_message>
dados: 2026-10-16 08:21 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/carteira_mensal/Out_2026.xlsx
+++ b/xlsx/carteira_mensal/Out_2026.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="89">
   <si>
     <t>Acompanhamento de Carteira</t>
   </si>
@@ -210,10 +210,37 @@
     <t>FERNANDA DOCHVAT SILVA</t>
   </si>
   <si>
+    <t>ADRIANA REGO BARROS MAGALHÃES</t>
+  </si>
+  <si>
+    <t>Porta</t>
+  </si>
+  <si>
+    <t>13/10/26</t>
+  </si>
+  <si>
+    <t>RAYSSA BARBOSA SILVA</t>
+  </si>
+  <si>
+    <t>15/10/26</t>
+  </si>
+  <si>
+    <t>VIVIAN MOURA BENIFICA GAZOLA</t>
+  </si>
+  <si>
+    <t>Já é cliente</t>
+  </si>
+  <si>
+    <t>Patrícia Santos da Silva</t>
+  </si>
+  <si>
+    <t>Fábrica</t>
+  </si>
+  <si>
     <t>Quantidade de Projetos</t>
   </si>
   <si>
-    <t>4</t>
+    <t>7</t>
   </si>
   <si>
     <t>Quantidade de Orçamentos</t>
@@ -222,22 +249,22 @@
     <t>Pontuação Total</t>
   </si>
   <si>
-    <t>1.92</t>
+    <t>1.93</t>
   </si>
   <si>
     <t>Valor Total Bruto</t>
   </si>
   <si>
-    <t>139.812,20</t>
-  </si>
-  <si>
-    <t>96.376,92</t>
+    <t>144.101,67</t>
+  </si>
+  <si>
+    <t>99.470,44</t>
   </si>
   <si>
     <t>Valor Total Líquido</t>
   </si>
   <si>
-    <t>91.189,24</t>
+    <t>94.282,76</t>
   </si>
   <si>
     <t>Total Líquido sem o Per</t>
@@ -252,7 +279,7 @@
     <t>Total Adicional dos Ambientes</t>
   </si>
   <si>
-    <t>4.690,05</t>
+    <t>5.050,05</t>
   </si>
 </sst>
 </file>
@@ -321,7 +348,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:O45"/>
+  <dimension ref="A2:O48"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="53.22265625" customWidth="true" bestFit="true"/>
@@ -759,76 +786,217 @@
         <v>61</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>65</v>
+      </c>
+      <c r="B35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1038.0</v>
+      </c>
+      <c r="D35" t="s">
+        <v>67</v>
+      </c>
+      <c r="E35" t="s">
+        <v>68</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G35" t="s">
+        <v>50</v>
+      </c>
+      <c r="H35" t="s">
+        <v>69</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1700.0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>1700.0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1700.0</v>
+      </c>
+      <c r="M35" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="N35" t="n">
+        <v>103801.0</v>
+      </c>
+      <c r="O35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" t="s">
+        <v>71</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1048.0</v>
+      </c>
+      <c r="D36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E36" t="s">
+        <v>60</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G36" t="s">
+        <v>50</v>
+      </c>
+      <c r="H36" t="s">
+        <v>69</v>
+      </c>
+      <c r="I36" t="n">
+        <v>340.52</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>340.52</v>
+      </c>
+      <c r="L36" t="n">
+        <v>340.52</v>
+      </c>
+      <c r="M36" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>104801.0</v>
+      </c>
+      <c r="O36" t="s">
+        <v>69</v>
+      </c>
+    </row>
     <row r="37">
-      <c r="A37" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B39" s="3" t="s">
+      <c r="A37" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" t="s">
+        <v>73</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1047.0</v>
+      </c>
+      <c r="D37" t="s">
+        <v>69</v>
+      </c>
+      <c r="E37" t="s">
+        <v>56</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G37" t="s">
+        <v>50</v>
+      </c>
+      <c r="H37" t="s">
+        <v>69</v>
+      </c>
+      <c r="I37" t="n">
+        <v>1053.0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1053.0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1053.0</v>
+      </c>
+      <c r="M37" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="N37" t="n">
+        <v>104701.0</v>
+      </c>
+      <c r="O37" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>17</v>
+        <v>76</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dados: 2026-10-20 08:21 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/carteira_mensal/Out_2026.xlsx
+++ b/xlsx/carteira_mensal/Out_2026.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="102">
   <si>
     <t>Acompanhamento de Carteira</t>
   </si>
@@ -225,6 +225,21 @@
     <t>15/10/26</t>
   </si>
   <si>
+    <t>REGINA RURIKO TATEIGI</t>
+  </si>
+  <si>
+    <t>14/10/26</t>
+  </si>
+  <si>
+    <t>Victor Costa</t>
+  </si>
+  <si>
+    <t>ESCRITÓRIO E DORMITÓRIO</t>
+  </si>
+  <si>
+    <t>19/10/26</t>
+  </si>
+  <si>
     <t>VIVIAN MOURA BENIFICA GAZOLA</t>
   </si>
   <si>
@@ -261,7 +276,7 @@
     <t>Quantidade de Projetos</t>
   </si>
   <si>
-    <t>10</t>
+    <t>11</t>
   </si>
   <si>
     <t>Quantidade de Orçamentos</t>
@@ -270,40 +285,40 @@
     <t>Pontuação Total</t>
   </si>
   <si>
-    <t>1.91</t>
+    <t>1.94</t>
   </si>
   <si>
     <t>Valor Total Bruto</t>
   </si>
   <si>
-    <t>226.245,62</t>
-  </si>
-  <si>
-    <t>157.481,60</t>
+    <t>265.448,92</t>
+  </si>
+  <si>
+    <t>187.181,60</t>
   </si>
   <si>
     <t>Valor Total Líquido</t>
   </si>
   <si>
-    <t>146.751,27</t>
+    <t>174.650,12</t>
   </si>
   <si>
     <t>Total Líquido sem o Per</t>
   </si>
   <si>
-    <t>145.666,64</t>
+    <t>173.565,49</t>
   </si>
   <si>
     <t>Total Diferença Financeira</t>
   </si>
   <si>
-    <t>10.730,33</t>
+    <t>12.531,48</t>
   </si>
   <si>
     <t>Total Adicional dos Ambientes</t>
   </si>
   <si>
-    <t>7.399,30</t>
+    <t>8.899,25</t>
   </si>
 </sst>
 </file>
@@ -372,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:O51"/>
+  <dimension ref="A2:O52"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="53.22265625" customWidth="true" bestFit="true"/>
@@ -862,63 +877,63 @@
         <v>70</v>
       </c>
       <c r="B36" t="s">
+        <v>47</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1044.0</v>
+      </c>
+      <c r="D36" t="s">
         <v>71</v>
       </c>
-      <c r="C36" t="n">
-        <v>1048.0</v>
-      </c>
-      <c r="D36" t="s">
-        <v>69</v>
-      </c>
       <c r="E36" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="F36" t="n">
         <v>1.0</v>
       </c>
       <c r="G36" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="H36" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="I36" t="n">
-        <v>340.52</v>
+        <v>29700.0</v>
       </c>
       <c r="J36" t="n">
-        <v>0.0</v>
+        <v>1801.15</v>
       </c>
       <c r="K36" t="n">
-        <v>340.52</v>
+        <v>27898.85</v>
       </c>
       <c r="L36" t="n">
-        <v>340.52</v>
+        <v>27898.85</v>
       </c>
       <c r="M36" t="n">
-        <v>3.0</v>
+        <v>2.1</v>
       </c>
       <c r="N36" t="n">
-        <v>104801.0</v>
+        <v>104401.0</v>
       </c>
       <c r="O36" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B37" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C37" t="n">
-        <v>1047.0</v>
+        <v>1048.0</v>
       </c>
       <c r="D37" t="s">
         <v>69</v>
       </c>
       <c r="E37" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F37" t="n">
         <v>1.0</v>
@@ -930,22 +945,22 @@
         <v>69</v>
       </c>
       <c r="I37" t="n">
-        <v>1053.0</v>
+        <v>340.52</v>
       </c>
       <c r="J37" t="n">
         <v>0.0</v>
       </c>
       <c r="K37" t="n">
-        <v>1053.0</v>
+        <v>340.52</v>
       </c>
       <c r="L37" t="n">
-        <v>1053.0</v>
+        <v>340.52</v>
       </c>
       <c r="M37" t="n">
-        <v>2.01</v>
+        <v>3.0</v>
       </c>
       <c r="N37" t="n">
-        <v>104701.0</v>
+        <v>104801.0</v>
       </c>
       <c r="O37" t="s">
         <v>69</v>
@@ -953,19 +968,19 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="C38" t="n">
-        <v>1050.0</v>
+        <v>1047.0</v>
       </c>
       <c r="D38" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E38" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F38" t="n">
         <v>1.0</v>
@@ -974,45 +989,45 @@
         <v>50</v>
       </c>
       <c r="H38" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="I38" t="n">
-        <v>1931.16</v>
+        <v>1053.0</v>
       </c>
       <c r="J38" t="n">
         <v>0.0</v>
       </c>
       <c r="K38" t="n">
-        <v>1931.16</v>
+        <v>1053.0</v>
       </c>
       <c r="L38" t="n">
-        <v>1931.16</v>
+        <v>1053.0</v>
       </c>
       <c r="M38" t="n">
-        <v>1.12</v>
+        <v>2.01</v>
       </c>
       <c r="N38" t="n">
-        <v>105001.0</v>
+        <v>104701.0</v>
       </c>
       <c r="O38" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B39" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="C39" t="n">
-        <v>1053.0</v>
+        <v>1050.0</v>
       </c>
       <c r="D39" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E39" t="s">
-        <v>79</v>
+        <v>49</v>
       </c>
       <c r="F39" t="n">
         <v>1.0</v>
@@ -1021,45 +1036,45 @@
         <v>50</v>
       </c>
       <c r="H39" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I39" t="n">
-        <v>5180.0</v>
+        <v>1931.16</v>
       </c>
       <c r="J39" t="n">
-        <v>376.9</v>
+        <v>0.0</v>
       </c>
       <c r="K39" t="n">
-        <v>4803.1</v>
+        <v>1931.16</v>
       </c>
       <c r="L39" t="n">
-        <v>4803.1</v>
+        <v>1931.16</v>
       </c>
       <c r="M39" t="n">
-        <v>1.98</v>
+        <v>1.12</v>
       </c>
       <c r="N39" t="n">
-        <v>105301.0</v>
+        <v>105001.0</v>
       </c>
       <c r="O39" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B40" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="C40" t="n">
-        <v>1051.0</v>
+        <v>1053.0</v>
       </c>
       <c r="D40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E40" t="s">
-        <v>56</v>
+        <v>84</v>
       </c>
       <c r="F40" t="n">
         <v>1.0</v>
@@ -1068,100 +1083,147 @@
         <v>50</v>
       </c>
       <c r="H40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="I40" t="n">
+        <v>5180.0</v>
+      </c>
+      <c r="J40" t="n">
+        <v>376.9</v>
+      </c>
+      <c r="K40" t="n">
+        <v>4803.1</v>
+      </c>
+      <c r="L40" t="n">
+        <v>4803.1</v>
+      </c>
+      <c r="M40" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="N40" t="n">
+        <v>105301.0</v>
+      </c>
+      <c r="O40" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>85</v>
+      </c>
+      <c r="B41" t="s">
+        <v>63</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1051.0</v>
+      </c>
+      <c r="D41" t="s">
+        <v>83</v>
+      </c>
+      <c r="E41" t="s">
+        <v>56</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G41" t="s">
+        <v>50</v>
+      </c>
+      <c r="H41" t="s">
+        <v>74</v>
+      </c>
+      <c r="I41" t="n">
         <v>50900.0</v>
       </c>
-      <c r="J40" t="n">
+      <c r="J41" t="n">
         <v>5165.75</v>
       </c>
-      <c r="K40" t="n">
+      <c r="K41" t="n">
         <v>45734.25</v>
       </c>
-      <c r="L40" t="n">
+      <c r="L41" t="n">
         <v>44649.62</v>
       </c>
-      <c r="M40" t="n">
+      <c r="M41" t="n">
         <v>1.93</v>
       </c>
-      <c r="N40" t="n">
+      <c r="N41" t="n">
         <v>105101.0</v>
       </c>
-      <c r="O40" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>82</v>
+      <c r="O41" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>17</v>
+        <v>91</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>89</v>
+        <v>17</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dados: 2026-10-22 08:21 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/carteira_mensal/Out_2026.xlsx
+++ b/xlsx/carteira_mensal/Out_2026.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="101">
   <si>
     <t>Acompanhamento de Carteira</t>
   </si>
@@ -156,7 +156,7 @@
     <t>Mariana Andrade Derossi</t>
   </si>
   <si>
-    <t>Cliente de porta</t>
+    <t>Porta</t>
   </si>
   <si>
     <t>17/09/26</t>
@@ -183,7 +183,7 @@
     <t>25/09/26</t>
   </si>
   <si>
-    <t>BIANCA RODRIGUES</t>
+    <t>bianca rodrigues</t>
   </si>
   <si>
     <t>CARLA EMÍLIA DE OLIVEIRA SOUZA FERREIRA</t>
@@ -211,9 +211,6 @@
   </si>
   <si>
     <t>ADRIANA REGO BARROS MAGALHÃES</t>
-  </si>
-  <si>
-    <t>Porta</t>
   </si>
   <si>
     <t>13/10/26</t>
@@ -830,16 +827,16 @@
         <v>65</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="C35" t="n">
         <v>1038.0</v>
       </c>
       <c r="D35" t="s">
+        <v>66</v>
+      </c>
+      <c r="E35" t="s">
         <v>67</v>
-      </c>
-      <c r="E35" t="s">
-        <v>68</v>
       </c>
       <c r="F35" t="n">
         <v>1.0</v>
@@ -848,7 +845,7 @@
         <v>50</v>
       </c>
       <c r="H35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I35" t="n">
         <v>1700.0</v>
@@ -869,12 +866,12 @@
         <v>103801.0</v>
       </c>
       <c r="O35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B36" t="s">
         <v>47</v>
@@ -883,19 +880,19 @@
         <v>1044.0</v>
       </c>
       <c r="D36" t="s">
+        <v>70</v>
+      </c>
+      <c r="E36" t="s">
         <v>71</v>
-      </c>
-      <c r="E36" t="s">
-        <v>72</v>
       </c>
       <c r="F36" t="n">
         <v>1.0</v>
       </c>
       <c r="G36" t="s">
+        <v>72</v>
+      </c>
+      <c r="H36" t="s">
         <v>73</v>
-      </c>
-      <c r="H36" t="s">
-        <v>74</v>
       </c>
       <c r="I36" t="n">
         <v>29700.0</v>
@@ -916,21 +913,21 @@
         <v>104401.0</v>
       </c>
       <c r="O36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
+        <v>74</v>
+      </c>
+      <c r="B37" t="s">
         <v>75</v>
-      </c>
-      <c r="B37" t="s">
-        <v>76</v>
       </c>
       <c r="C37" t="n">
         <v>1048.0</v>
       </c>
       <c r="D37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E37" t="s">
         <v>60</v>
@@ -942,7 +939,7 @@
         <v>50</v>
       </c>
       <c r="H37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I37" t="n">
         <v>340.52</v>
@@ -963,21 +960,21 @@
         <v>104801.0</v>
       </c>
       <c r="O37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
+        <v>76</v>
+      </c>
+      <c r="B38" t="s">
         <v>77</v>
-      </c>
-      <c r="B38" t="s">
-        <v>78</v>
       </c>
       <c r="C38" t="n">
         <v>1047.0</v>
       </c>
       <c r="D38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E38" t="s">
         <v>56</v>
@@ -989,7 +986,7 @@
         <v>50</v>
       </c>
       <c r="H38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I38" t="n">
         <v>1053.0</v>
@@ -1010,12 +1007,12 @@
         <v>104701.0</v>
       </c>
       <c r="O38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B39" t="s">
         <v>58</v>
@@ -1024,7 +1021,7 @@
         <v>1050.0</v>
       </c>
       <c r="D39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E39" t="s">
         <v>49</v>
@@ -1036,7 +1033,7 @@
         <v>50</v>
       </c>
       <c r="H39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I39" t="n">
         <v>1931.16</v>
@@ -1057,24 +1054,24 @@
         <v>105001.0</v>
       </c>
       <c r="O39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
+        <v>80</v>
+      </c>
+      <c r="B40" t="s">
         <v>81</v>
-      </c>
-      <c r="B40" t="s">
-        <v>82</v>
       </c>
       <c r="C40" t="n">
         <v>1053.0</v>
       </c>
       <c r="D40" t="s">
+        <v>82</v>
+      </c>
+      <c r="E40" t="s">
         <v>83</v>
-      </c>
-      <c r="E40" t="s">
-        <v>84</v>
       </c>
       <c r="F40" t="n">
         <v>1.0</v>
@@ -1083,7 +1080,7 @@
         <v>50</v>
       </c>
       <c r="H40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I40" t="n">
         <v>5180.0</v>
@@ -1104,12 +1101,12 @@
         <v>105301.0</v>
       </c>
       <c r="O40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B41" t="s">
         <v>63</v>
@@ -1118,7 +1115,7 @@
         <v>1051.0</v>
       </c>
       <c r="D41" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E41" t="s">
         <v>56</v>
@@ -1130,7 +1127,7 @@
         <v>50</v>
       </c>
       <c r="H41" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I41" t="n">
         <v>50900.0</v>
@@ -1151,39 +1148,39 @@
         <v>105101.0</v>
       </c>
       <c r="O41" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B46" s="3" t="s">
         <v>89</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>91</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="48">
@@ -1191,39 +1188,39 @@
         <v>17</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B49" s="3" t="s">
         <v>94</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B50" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B51" s="3" t="s">
         <v>98</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B52" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dados: 2026-10-25 08:20 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/carteira_mensal/Out_2026.xlsx
+++ b/xlsx/carteira_mensal/Out_2026.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="107">
   <si>
     <t>Acompanhamento de Carteira</t>
   </si>
@@ -270,10 +270,28 @@
     <t>Claudio Wasserman</t>
   </si>
   <si>
+    <t>Willian Rodrigues Lima</t>
+  </si>
+  <si>
+    <t>Indicação de Amigo</t>
+  </si>
+  <si>
+    <t>21/10/26</t>
+  </si>
+  <si>
+    <t>24/10/26</t>
+  </si>
+  <si>
+    <t>DANIELA IDA MENEGATTI MILANO</t>
+  </si>
+  <si>
+    <t>23/10/26</t>
+  </si>
+  <si>
     <t>Quantidade de Projetos</t>
   </si>
   <si>
-    <t>11</t>
+    <t>13</t>
   </si>
   <si>
     <t>Quantidade de Orçamentos</t>
@@ -282,40 +300,40 @@
     <t>Pontuação Total</t>
   </si>
   <si>
-    <t>1.94</t>
+    <t>1.93</t>
   </si>
   <si>
     <t>Valor Total Bruto</t>
   </si>
   <si>
-    <t>265.448,92</t>
-  </si>
-  <si>
-    <t>187.181,60</t>
+    <t>328.439,51</t>
+  </si>
+  <si>
+    <t>237.024,72</t>
   </si>
   <si>
     <t>Valor Total Líquido</t>
   </si>
   <si>
-    <t>174.650,12</t>
+    <t>215.453,03</t>
   </si>
   <si>
     <t>Total Líquido sem o Per</t>
   </si>
   <si>
-    <t>173.565,49</t>
+    <t>214.368,40</t>
   </si>
   <si>
     <t>Total Diferença Financeira</t>
   </si>
   <si>
-    <t>12.531,48</t>
+    <t>21.571,69</t>
   </si>
   <si>
     <t>Total Adicional dos Ambientes</t>
   </si>
   <si>
-    <t>8.899,25</t>
+    <t>11.185,10</t>
   </si>
 </sst>
 </file>
@@ -384,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:O52"/>
+  <dimension ref="A2:O54"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="53.22265625" customWidth="true" bestFit="true"/>
@@ -1151,76 +1169,170 @@
         <v>82</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2" t="s">
+    <row r="42">
+      <c r="A42" t="s">
         <v>85</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B42" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="s">
+      <c r="C42" t="n">
+        <v>1055.0</v>
+      </c>
+      <c r="D42" t="s">
         <v>87</v>
       </c>
-      <c r="B45" s="3" t="s">
-        <v>86</v>
+      <c r="E42" t="s">
+        <v>83</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G42" t="s">
+        <v>50</v>
+      </c>
+      <c r="H42" t="s">
+        <v>88</v>
+      </c>
+      <c r="I42" t="n">
+        <v>36000.0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>7260.81</v>
+      </c>
+      <c r="K42" t="n">
+        <v>28739.19</v>
+      </c>
+      <c r="L42" t="n">
+        <v>28739.19</v>
+      </c>
+      <c r="M42" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="N42" t="n">
+        <v>105501.0</v>
+      </c>
+      <c r="O42" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>89</v>
+      </c>
+      <c r="B43" t="s">
+        <v>58</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1057.0</v>
+      </c>
+      <c r="D43" t="s">
+        <v>90</v>
+      </c>
+      <c r="E43" t="s">
+        <v>56</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G43" t="s">
+        <v>50</v>
+      </c>
+      <c r="H43" t="s">
+        <v>88</v>
+      </c>
+      <c r="I43" t="n">
+        <v>13843.12</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1779.4</v>
+      </c>
+      <c r="K43" t="n">
+        <v>12063.72</v>
+      </c>
+      <c r="L43" t="n">
+        <v>12063.72</v>
+      </c>
+      <c r="M43" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="N43" t="n">
+        <v>105701.0</v>
+      </c>
+      <c r="O43" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>17</v>
+        <v>94</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="s">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dados: 2026-10-29 08:21 (131 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/carteira_mensal/Out_2026.xlsx
+++ b/xlsx/carteira_mensal/Out_2026.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="105">
   <si>
     <t>Acompanhamento de Carteira</t>
   </si>
@@ -222,54 +222,42 @@
     <t>15/10/26</t>
   </si>
   <si>
-    <t>REGINA RURIKO TATEIGI</t>
-  </si>
-  <si>
-    <t>14/10/26</t>
-  </si>
-  <si>
-    <t>Victor Costa</t>
-  </si>
-  <si>
-    <t>ESCRITÓRIO E DORMITÓRIO</t>
+    <t>VIVIAN MOURA BENIFICA GAZOLA</t>
+  </si>
+  <si>
+    <t>Já é cliente</t>
+  </si>
+  <si>
+    <t>Patrícia Santos da Silva</t>
+  </si>
+  <si>
+    <t>Fábrica</t>
+  </si>
+  <si>
+    <t>Patricia Souza Fernandez</t>
+  </si>
+  <si>
+    <t>16/10/26</t>
+  </si>
+  <si>
+    <t>Elaine Massumi Higashi</t>
+  </si>
+  <si>
+    <t>Parceiro</t>
+  </si>
+  <si>
+    <t>17/10/26</t>
+  </si>
+  <si>
+    <t>ERIC SERPA</t>
+  </si>
+  <si>
+    <t>Claudio Wasserman</t>
   </si>
   <si>
     <t>19/10/26</t>
   </si>
   <si>
-    <t>VIVIAN MOURA BENIFICA GAZOLA</t>
-  </si>
-  <si>
-    <t>Já é cliente</t>
-  </si>
-  <si>
-    <t>Patrícia Santos da Silva</t>
-  </si>
-  <si>
-    <t>Fábrica</t>
-  </si>
-  <si>
-    <t>Patricia Souza Fernandez</t>
-  </si>
-  <si>
-    <t>16/10/26</t>
-  </si>
-  <si>
-    <t>Elaine Massumi Higashi</t>
-  </si>
-  <si>
-    <t>Parceiro</t>
-  </si>
-  <si>
-    <t>17/10/26</t>
-  </si>
-  <si>
-    <t>ERIC SERPA</t>
-  </si>
-  <si>
-    <t>Claudio Wasserman</t>
-  </si>
-  <si>
     <t>Willian Rodrigues Lima</t>
   </si>
   <si>
@@ -288,6 +276,12 @@
     <t>23/10/26</t>
   </si>
   <si>
+    <t>26/10/26</t>
+  </si>
+  <si>
+    <t>28/10/26</t>
+  </si>
+  <si>
     <t>Quantidade de Projetos</t>
   </si>
   <si>
@@ -300,40 +294,40 @@
     <t>Pontuação Total</t>
   </si>
   <si>
-    <t>1.93</t>
+    <t>1.91</t>
   </si>
   <si>
     <t>Valor Total Bruto</t>
   </si>
   <si>
-    <t>328.439,51</t>
-  </si>
-  <si>
-    <t>237.024,72</t>
+    <t>315.779,97</t>
+  </si>
+  <si>
+    <t>226.658,31</t>
   </si>
   <si>
     <t>Valor Total Líquido</t>
   </si>
   <si>
-    <t>215.453,03</t>
+    <t>204.925,66</t>
   </si>
   <si>
     <t>Total Líquido sem o Per</t>
   </si>
   <si>
-    <t>214.368,40</t>
+    <t>203.841,03</t>
   </si>
   <si>
     <t>Total Diferença Financeira</t>
   </si>
   <si>
-    <t>21.571,69</t>
+    <t>21.732,65</t>
   </si>
   <si>
     <t>Total Adicional dos Ambientes</t>
   </si>
   <si>
-    <t>11.185,10</t>
+    <t>10.512,36</t>
   </si>
 </sst>
 </file>
@@ -892,63 +886,63 @@
         <v>69</v>
       </c>
       <c r="B36" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="C36" t="n">
-        <v>1044.0</v>
+        <v>1048.0</v>
       </c>
       <c r="D36" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E36" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="F36" t="n">
         <v>1.0</v>
       </c>
       <c r="G36" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="H36" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="I36" t="n">
-        <v>29700.0</v>
+        <v>340.52</v>
       </c>
       <c r="J36" t="n">
-        <v>1801.15</v>
+        <v>0.0</v>
       </c>
       <c r="K36" t="n">
-        <v>27898.85</v>
+        <v>340.52</v>
       </c>
       <c r="L36" t="n">
-        <v>27898.85</v>
+        <v>340.52</v>
       </c>
       <c r="M36" t="n">
-        <v>2.1</v>
+        <v>3.0</v>
       </c>
       <c r="N36" t="n">
-        <v>104401.0</v>
+        <v>104801.0</v>
       </c>
       <c r="O36" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C37" t="n">
-        <v>1048.0</v>
+        <v>1047.0</v>
       </c>
       <c r="D37" t="s">
         <v>68</v>
       </c>
       <c r="E37" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F37" t="n">
         <v>1.0</v>
@@ -960,22 +954,22 @@
         <v>68</v>
       </c>
       <c r="I37" t="n">
-        <v>340.52</v>
+        <v>1053.0</v>
       </c>
       <c r="J37" t="n">
         <v>0.0</v>
       </c>
       <c r="K37" t="n">
-        <v>340.52</v>
+        <v>1053.0</v>
       </c>
       <c r="L37" t="n">
-        <v>340.52</v>
+        <v>1053.0</v>
       </c>
       <c r="M37" t="n">
-        <v>3.0</v>
+        <v>2.01</v>
       </c>
       <c r="N37" t="n">
-        <v>104801.0</v>
+        <v>104701.0</v>
       </c>
       <c r="O37" t="s">
         <v>68</v>
@@ -983,19 +977,19 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B38" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="C38" t="n">
-        <v>1047.0</v>
+        <v>1050.0</v>
       </c>
       <c r="D38" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="E38" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="F38" t="n">
         <v>1.0</v>
@@ -1004,45 +998,45 @@
         <v>50</v>
       </c>
       <c r="H38" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I38" t="n">
-        <v>1053.0</v>
+        <v>1931.16</v>
       </c>
       <c r="J38" t="n">
         <v>0.0</v>
       </c>
       <c r="K38" t="n">
-        <v>1053.0</v>
+        <v>1931.16</v>
       </c>
       <c r="L38" t="n">
-        <v>1053.0</v>
+        <v>1931.16</v>
       </c>
       <c r="M38" t="n">
-        <v>2.01</v>
+        <v>1.12</v>
       </c>
       <c r="N38" t="n">
-        <v>104701.0</v>
+        <v>105001.0</v>
       </c>
       <c r="O38" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1053.0</v>
+      </c>
+      <c r="D39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E39" t="s">
         <v>78</v>
-      </c>
-      <c r="B39" t="s">
-        <v>58</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1050.0</v>
-      </c>
-      <c r="D39" t="s">
-        <v>79</v>
-      </c>
-      <c r="E39" t="s">
-        <v>49</v>
       </c>
       <c r="F39" t="n">
         <v>1.0</v>
@@ -1051,45 +1045,45 @@
         <v>50</v>
       </c>
       <c r="H39" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I39" t="n">
-        <v>1931.16</v>
+        <v>5180.0</v>
       </c>
       <c r="J39" t="n">
-        <v>0.0</v>
+        <v>376.9</v>
       </c>
       <c r="K39" t="n">
-        <v>1931.16</v>
+        <v>4803.1</v>
       </c>
       <c r="L39" t="n">
-        <v>1931.16</v>
+        <v>4803.1</v>
       </c>
       <c r="M39" t="n">
-        <v>1.12</v>
+        <v>1.98</v>
       </c>
       <c r="N39" t="n">
-        <v>105001.0</v>
+        <v>105301.0</v>
       </c>
       <c r="O39" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B40" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="C40" t="n">
-        <v>1053.0</v>
+        <v>1051.0</v>
       </c>
       <c r="D40" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E40" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="F40" t="n">
         <v>1.0</v>
@@ -1098,45 +1092,45 @@
         <v>50</v>
       </c>
       <c r="H40" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I40" t="n">
-        <v>5180.0</v>
+        <v>50900.0</v>
       </c>
       <c r="J40" t="n">
-        <v>376.9</v>
+        <v>5165.75</v>
       </c>
       <c r="K40" t="n">
-        <v>4803.1</v>
+        <v>45734.25</v>
       </c>
       <c r="L40" t="n">
-        <v>4803.1</v>
+        <v>44649.62</v>
       </c>
       <c r="M40" t="n">
-        <v>1.98</v>
+        <v>1.93</v>
       </c>
       <c r="N40" t="n">
-        <v>105301.0</v>
+        <v>105101.0</v>
       </c>
       <c r="O40" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B41" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="C41" t="n">
-        <v>1051.0</v>
+        <v>1055.0</v>
       </c>
       <c r="D41" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E41" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="F41" t="n">
         <v>1.0</v>
@@ -1145,28 +1139,28 @@
         <v>50</v>
       </c>
       <c r="H41" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="I41" t="n">
-        <v>50900.0</v>
+        <v>36000.0</v>
       </c>
       <c r="J41" t="n">
-        <v>5165.75</v>
+        <v>7260.81</v>
       </c>
       <c r="K41" t="n">
-        <v>45734.25</v>
+        <v>28739.19</v>
       </c>
       <c r="L41" t="n">
-        <v>44649.62</v>
+        <v>28739.19</v>
       </c>
       <c r="M41" t="n">
-        <v>1.93</v>
+        <v>1.9</v>
       </c>
       <c r="N41" t="n">
-        <v>105101.0</v>
+        <v>105501.0</v>
       </c>
       <c r="O41" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42">
@@ -1174,16 +1168,16 @@
         <v>85</v>
       </c>
       <c r="B42" t="s">
+        <v>58</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1057.0</v>
+      </c>
+      <c r="D42" t="s">
         <v>86</v>
       </c>
-      <c r="C42" t="n">
-        <v>1055.0</v>
-      </c>
-      <c r="D42" t="s">
-        <v>87</v>
-      </c>
       <c r="E42" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="F42" t="n">
         <v>1.0</v>
@@ -1192,42 +1186,42 @@
         <v>50</v>
       </c>
       <c r="H42" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I42" t="n">
-        <v>36000.0</v>
+        <v>13843.12</v>
       </c>
       <c r="J42" t="n">
-        <v>7260.81</v>
+        <v>1779.4</v>
       </c>
       <c r="K42" t="n">
-        <v>28739.19</v>
+        <v>12063.72</v>
       </c>
       <c r="L42" t="n">
-        <v>28739.19</v>
+        <v>12063.72</v>
       </c>
       <c r="M42" t="n">
         <v>1.9</v>
       </c>
       <c r="N42" t="n">
-        <v>105501.0</v>
+        <v>105701.0</v>
       </c>
       <c r="O42" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="B43" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C43" t="n">
-        <v>1057.0</v>
+        <v>1060.0</v>
       </c>
       <c r="D43" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E43" t="s">
         <v>56</v>
@@ -1242,22 +1236,22 @@
         <v>88</v>
       </c>
       <c r="I43" t="n">
-        <v>13843.12</v>
+        <v>19333.59</v>
       </c>
       <c r="J43" t="n">
-        <v>1779.4</v>
+        <v>1962.11</v>
       </c>
       <c r="K43" t="n">
-        <v>12063.72</v>
+        <v>17371.48</v>
       </c>
       <c r="L43" t="n">
-        <v>12063.72</v>
+        <v>17371.48</v>
       </c>
       <c r="M43" t="n">
-        <v>1.9</v>
+        <v>1.93</v>
       </c>
       <c r="N43" t="n">
-        <v>105701.0</v>
+        <v>106001.0</v>
       </c>
       <c r="O43" t="s">
         <v>88</v>
@@ -1265,34 +1259,34 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50">
@@ -1300,39 +1294,39 @@
         <v>17</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>